<commit_message>
corrigido decontos incorretos em controle
</commit_message>
<xml_diff>
--- a/base/database.xlsx
+++ b/base/database.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\eliasgk\Documents\Python Projects\RelatorioCelesc\base\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Program Files (x86)\oab-programas\RelatorioCelesc\base\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F1D44A7-2AB8-4145-B35E-F46203F47A38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9BCBCD2-3EDA-47E0-851A-2A601BAFFA52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-20610" yWindow="1335" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="116">
   <si>
     <t>UC</t>
   </si>
@@ -367,6 +367,12 @@
   </si>
   <si>
     <t>Campos Novos</t>
+  </si>
+  <si>
+    <t>230</t>
+  </si>
+  <si>
+    <t>0059180801</t>
   </si>
 </sst>
 </file>
@@ -1157,8 +1163,8 @@
       <c r="A38" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="B38" s="5">
-        <v>227</v>
+      <c r="B38" s="5" t="s">
+        <v>114</v>
       </c>
       <c r="C38" s="5" t="s">
         <v>104</v>
@@ -1440,8 +1446,15 @@
       </c>
     </row>
     <row r="64" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A64" s="2"/>
-      <c r="C64" s="5"/>
+      <c r="A64" s="2" t="s">
+        <v>115</v>
+      </c>
+      <c r="B64" s="1">
+        <v>208</v>
+      </c>
+      <c r="C64" s="5" t="s">
+        <v>10</v>
+      </c>
     </row>
     <row r="65" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A65" s="2"/>

</xml_diff>